<commit_message>
fix: improve bulk registration cancellation and payment handling logic
</commit_message>
<xml_diff>
--- a/Template-Pendaftaran-Kolektif-Trailrun-Jiwandana.xlsx
+++ b/Template-Pendaftaran-Kolektif-Trailrun-Jiwandana.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:P11"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -415,7 +415,6 @@
     <col min="14" max="14" width="18.83203125" customWidth="1"/>
     <col min="15" max="15" width="30.83203125" customWidth="1"/>
     <col min="16" max="16" width="28.83203125" customWidth="1"/>
-    <col min="17" max="17" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,9 +464,6 @@
         <v>Kontak Darurat (Nama &amp; No HP) *</v>
       </c>
       <c r="P1" t="str">
-        <v>Nama Komunitas / Running Club</v>
-      </c>
-      <c r="Q1" t="str">
         <v>Riwayat Medis (Opsional)</v>
       </c>
     </row>
@@ -476,7 +472,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Budi Santoso</v>
+        <v>Test 1</v>
       </c>
       <c r="C2" t="str">
         <v>3516011708950001</v>
@@ -518,9 +514,6 @@
         <v>Siti Aminah (081298765432)</v>
       </c>
       <c r="P2" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q2" t="str">
         <v>Tidak ada riwayat medis</v>
       </c>
     </row>
@@ -529,7 +522,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Dewi Lestari</v>
+        <v>Test 2</v>
       </c>
       <c r="C3" t="str">
         <v>3516016311980002</v>
@@ -571,9 +564,6 @@
         <v>Agus Santoso (081333444555)</v>
       </c>
       <c r="P3" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q3" t="str">
         <v>-</v>
       </c>
     </row>
@@ -582,7 +572,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Rizky Pratama</v>
+        <v>Test 3</v>
       </c>
       <c r="C4" t="str">
         <v>3578011004920003</v>
@@ -624,9 +614,6 @@
         <v>Rina Maya (085699887766)</v>
       </c>
       <c r="P4" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q4" t="str">
         <v>-</v>
       </c>
     </row>
@@ -635,7 +622,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Siti Nurhaliza</v>
+        <v>Test 4</v>
       </c>
       <c r="C5" t="str">
         <v>3516024505960004</v>
@@ -677,9 +664,6 @@
         <v>Ahmad Fauzi (082199887711)</v>
       </c>
       <c r="P5" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q5" t="str">
         <v>-</v>
       </c>
     </row>
@@ -688,7 +672,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Dimas Anggara</v>
+        <v>Test 5</v>
       </c>
       <c r="C6" t="str">
         <v>3578021209930005</v>
@@ -730,9 +714,6 @@
         <v>Wulandari (087888776622)</v>
       </c>
       <c r="P6" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q6" t="str">
         <v>-</v>
       </c>
     </row>
@@ -741,7 +722,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Rina Wulandari</v>
+        <v>Test 6</v>
       </c>
       <c r="C7" t="str">
         <v>3516035402970006</v>
@@ -783,9 +764,6 @@
         <v>Hendra Setiawan (081999887733)</v>
       </c>
       <c r="P7" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q7" t="str">
         <v>-</v>
       </c>
     </row>
@@ -794,7 +772,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>Fajar Hidayat</v>
+        <v>Test 7</v>
       </c>
       <c r="C8" t="str">
         <v>3515012001940007</v>
@@ -836,9 +814,6 @@
         <v>Ratna Sari (082299887744)</v>
       </c>
       <c r="P8" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q8" t="str">
         <v>-</v>
       </c>
     </row>
@@ -847,7 +822,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Anisa Rahmawati</v>
+        <v>Test 8</v>
       </c>
       <c r="C9" t="str">
         <v>3515026207990008</v>
@@ -889,9 +864,6 @@
         <v>Bambang Irawan (085799887755)</v>
       </c>
       <c r="P9" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q9" t="str">
         <v>-</v>
       </c>
     </row>
@@ -900,7 +872,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Bayu Kurniawan</v>
+        <v>Test 9</v>
       </c>
       <c r="C10" t="str">
         <v>3573010503910009</v>
@@ -942,9 +914,6 @@
         <v>Mega Utami (081288776666)</v>
       </c>
       <c r="P10" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q10" t="str">
         <v>-</v>
       </c>
     </row>
@@ -953,7 +922,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Fitri Handayani</v>
+        <v>Test 10</v>
       </c>
       <c r="C11" t="str">
         <v>3573024810950010</v>
@@ -995,15 +964,12 @@
         <v>Dedi Prasetyo (081399887777)</v>
       </c>
       <c r="P11" t="str">
-        <v>Pawitra Trail Runners</v>
-      </c>
-      <c r="Q11" t="str">
         <v>-</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>